<commit_message>
환율 2주 추가 (2026.04.26~05.09)
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260506.xlsx
+++ b/RNR_수입원가_2026_20260506.xlsx
@@ -14,9 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="환율" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="FxRateTable">환율!$A$7:$D$34</definedName>
     <definedName name="RemitTable1">외화송금내역!$A$3:$L$34</definedName>
     <definedName name="RemitTable2">외화송금내역!$A$37:$L$74</definedName>
+    <definedName name="FxRateTable">환율!$A$7:$D$37</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -16096,7 +16096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="15" customWidth="1" style="40" min="1" max="2"/>
@@ -16631,6 +16631,38 @@
       </c>
       <c r="D35" s="7" t="n">
         <v>1479.34</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="144" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B36" s="144" t="n">
+        <v>46144</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>1476.92</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="144" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B37" s="144" t="n">
+        <v>46151</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>1476.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EPO18 vendor 정정: Elicent → MAICO Italia (PROFORMA 근거)
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260506.xlsx
+++ b/RNR_수입원가_2026_20260506.xlsx
@@ -4949,12 +4949,12 @@
       </c>
       <c r="C31" s="78" t="inlineStr">
         <is>
-          <t>Elicent</t>
+          <t>MAICO Italia</t>
         </is>
       </c>
       <c r="D31" s="78" t="inlineStr">
         <is>
-          <t>T/T (EUR)</t>
+          <t>100% TT in advance</t>
         </is>
       </c>
       <c r="E31" s="78" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="N31" s="78" t="inlineStr">
         <is>
-          <t>AXC 200 ELICENT 60ea (EUR / 재고)</t>
+          <t>AXC 200 ELICENT VENTILATORE/FAN (60EA, EUR)</t>
         </is>
       </c>
       <c r="O31" s="149" t="n"/>
@@ -12061,7 +12061,7 @@
       </c>
       <c r="C32" s="103" t="inlineStr">
         <is>
-          <t>Elicent (EUR)</t>
+          <t>MAICO Italia (EUR)</t>
         </is>
       </c>
       <c r="D32" s="102" t="inlineStr">
@@ -14002,7 +14002,7 @@
       </c>
       <c r="C70" s="103" t="inlineStr">
         <is>
-          <t>Elicent</t>
+          <t>MAICO Italia</t>
         </is>
       </c>
       <c r="D70" s="104" t="n">

</xml_diff>